<commit_message>
WIP: la po no me responnnnnnnnnnnnnnnnnde MAS
</commit_message>
<xml_diff>
--- a/exports/no-tariff-classes-analysis.xlsx
+++ b/exports/no-tariff-classes-analysis.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Matches Excel" sheetId="6" r:id="rId6"/>
     <sheet name="Diagnóstico" sheetId="7" r:id="rId7"/>
     <sheet name="Metadata" sheetId="8" r:id="rId8"/>
+    <sheet name="Mappings confirmados" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -409,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:R9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,6 +449,24 @@
       <c r="L1" t="str">
         <v>Matches Excel</v>
       </c>
+      <c r="M1" t="str">
+        <v>Mapping confirmado</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Nombre/s histórico/s confirmado/s</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Política tarifaria</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Tarifa base confirmada</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Motivo mapping</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Matches mapping</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -469,10 +488,10 @@
         <v>2026-08-28</v>
       </c>
       <c r="G2" t="str">
-        <v>NO_SOURCE_EVIDENCE</v>
+        <v>CONFIRMED_MAPPING</v>
       </c>
       <c r="H2" t="str">
-        <v>No se encontró evidencia directa suficiente en las fuentes analizadas.</v>
+        <v>PO confirmó que S&amp;B Parejas corresponde a Salsa y Bachata en Pareja.</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -484,6 +503,24 @@
         <v>0</v>
       </c>
       <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Salsa y Bachata en Pareja | Salsa Y Bachata En Pareja | Salsa Y Bachata En Pareja _Fabi</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>PO confirmó que S&amp;B Parejas corresponde a Salsa y Bachata en Pareja.</v>
+      </c>
+      <c r="R2">
         <v>0</v>
       </c>
     </row>
@@ -507,21 +544,39 @@
         <v>2026-08-28</v>
       </c>
       <c r="G3" t="str">
-        <v>NO_SOURCE_EVIDENCE</v>
+        <v>CONFIRMED_HISTORICAL_ACTIVITY</v>
       </c>
       <c r="H3" t="str">
-        <v>No se encontró evidencia directa suficiente en las fuentes analizadas.</v>
+        <v>PO confirmó que corresponde a la clase de Kizomba de Fabi y utilizaba la cuota base general de la academia.</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" t="str">
+        <v>HISTORICAL_ACTIVITY</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Kizomba | Clase Kizomba</v>
+      </c>
+      <c r="O3" t="str">
+        <v>GENERAL_ACADEMY_RATE</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>PO confirmó que corresponde a la clase de Kizomba de Fabi y utilizaba la cuota base general de la academia.</v>
+      </c>
+      <c r="R3">
         <v>0</v>
       </c>
     </row>
@@ -545,10 +600,10 @@
         <v>2026-08-28</v>
       </c>
       <c r="G4" t="str">
-        <v>NO_SOURCE_EVIDENCE</v>
+        <v>CONFIRMED_MAPPING</v>
       </c>
       <c r="H4" t="str">
-        <v>No se encontró evidencia directa suficiente en las fuentes analizadas.</v>
+        <v>PO confirmó que Hells es un error de escritura y corresponde a Heels.</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -560,6 +615,24 @@
         <v>0</v>
       </c>
       <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Heels</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>PO confirmó que Hells es un error de escritura y corresponde a Heels.</v>
+      </c>
+      <c r="R4">
         <v>0</v>
       </c>
     </row>
@@ -583,10 +656,10 @@
         <v>2026-08-28</v>
       </c>
       <c r="G5" t="str">
-        <v>SPECIAL_PROGRAM_REVIEW</v>
+        <v>CONFIRMED_SPECIAL_PROGRAM</v>
       </c>
       <c r="H5" t="str">
-        <v>El nombre sugiere una formación/programa especial. Conviene revisar su esquema de cobro antes de crear una tarifa mensual estándar.</v>
+        <v>PO confirmó que la formación comenzó en abril de 2026, termina en diciembre de 2026 y tiene cuota base mensual de $90.000. Los valores $76.500, $72.000 y becas son condiciones particulares.</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -595,10 +668,28 @@
         <v>2</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>15</v>
+      </c>
+      <c r="M5" t="str">
+        <v>SPECIAL_PROGRAM</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Formacion Docente En Ritmos Caribeños Y Kizomba | Formación Docente En Ritmos Caribeños Y Kizomba</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>90000.00</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>PO confirmó que la formación comenzó en abril de 2026, termina en diciembre de 2026 y tiene cuota base mensual de $90.000. Los valores $76.500, $72.000 y becas son condiciones particulares.</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -621,22 +712,40 @@
         <v>2026-08-28</v>
       </c>
       <c r="G6" t="str">
-        <v>WORKBOOK_EVIDENCE_ONLY</v>
+        <v>CONFIRMED_MAPPING</v>
       </c>
       <c r="H6" t="str">
-        <v>Hay coincidencias en el Excel histórico, pero no existe una asociación directa con una tarifa final.</v>
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>40</v>
+      </c>
+      <c r="M6" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Coreográfico Femenino | Coreografico Femenino | Estilo Femenino</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+      <c r="R6">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -659,22 +768,40 @@
         <v>2026-02-01</v>
       </c>
       <c r="G7" t="str">
-        <v>WORKBOOK_EVIDENCE_ONLY</v>
+        <v>CONFIRMED_HISTORICAL_ACTIVITY</v>
       </c>
       <c r="H7" t="str">
-        <v>Hay coincidencias en el Excel histórico, pero no existe una asociación directa con una tarifa final.</v>
+        <v>PO confirmó que era una actividad independiente, utilizaba la cuota general y posteriormente pasó a llamarse Urban Flow.</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>10</v>
+      </c>
+      <c r="M7" t="str">
+        <v>HISTORICAL_ACTIVITY</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Coreografico E Masc Bachata Urban | Coreográfico E Masc Bachata Urban | Coreografico E.Masc-Bachata/Urban</v>
+      </c>
+      <c r="O7" t="str">
+        <v>GENERAL_ACADEMY_RATE</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>PO confirmó que era una actividad independiente, utilizaba la cuota general y posteriormente pasó a llamarse Urban Flow.</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -697,10 +824,10 @@
         <v>2026-08-21</v>
       </c>
       <c r="G8" t="str">
-        <v>NO_SOURCE_EVIDENCE</v>
+        <v>TEST_CLASS</v>
       </c>
       <c r="H8" t="str">
-        <v>No se encontró evidencia directa suficiente en las fuentes analizadas.</v>
+        <v>Clase de prueba. No corresponde reconstruir tarifas históricas y será eliminada posteriormente.</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -712,6 +839,24 @@
         <v>0</v>
       </c>
       <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" t="str">
+        <v>TEST_CLASS</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>Clase de prueba. No corresponde reconstruir tarifas históricas y será eliminada posteriormente.</v>
+      </c>
+      <c r="R8">
         <v>0</v>
       </c>
     </row>
@@ -735,10 +880,10 @@
         <v>2025-07-01</v>
       </c>
       <c r="G9" t="str">
-        <v>POSSIBLE_ALIAS</v>
+        <v>CONFIRMED_SPECIAL_PROGRAM</v>
       </c>
       <c r="H9" t="str">
-        <v>Hay otra actividad o clase con un nombre suficientemente similar como para revisar un posible mapping histórico.</v>
+        <v>PO confirmó que era un programa diferente de Tango regular, con cuota mensual de $70.000 y actualmente está dado de baja.</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -752,10 +897,28 @@
       <c r="L9">
         <v>40</v>
       </c>
+      <c r="M9" t="str">
+        <v>SPECIAL_PROGRAM</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Inst Sup Coreografico Tango 18 Meses | Inst.Sup.Coreografico -Tango /18 Meses | Instituto Superior Coreografico Tango 18 Meses</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v>70000.00</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>PO confirmó que era un programa diferente de Tango regular, con cuota mensual de $70.000 y actualmente está dado de baja.</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3276,7 +3439,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3318,25 +3481,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Clase kizomba</v>
+        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
       </c>
       <c r="B2">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="C2" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Ritmos Caribeños y Kizomba Parejas</v>
       </c>
       <c r="D2" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Ritmos latinos y caribeños</v>
       </c>
       <c r="E2" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
+        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
       </c>
       <c r="F2" t="str">
-        <v>Coreográfico Femenino</v>
+        <v>Ritmos Caribeños y Kizomba Parejas</v>
       </c>
       <c r="G2" t="str">
-        <v>SOFIA</v>
+        <v>FABI</v>
       </c>
       <c r="H2" t="str">
         <v>OK</v>
@@ -3350,31 +3513,28 @@
       <c r="K2" t="str">
         <v>2025-02-28</v>
       </c>
-      <c r="L2" t="str">
-        <v>La academia confirmó tarifa general de $15.000 para febrero de 2025. En marzo cambió a $20.000.</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Clase kizomba</v>
+        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
       </c>
       <c r="B3">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="C3" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Ritmos Caribeños y Kizomba Parejas</v>
       </c>
       <c r="D3" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Ritmos latinos y caribeños</v>
       </c>
       <c r="E3" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
+        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
       </c>
       <c r="F3" t="str">
-        <v>Coreográfico Femenino</v>
+        <v>Ritmos Caribeños y Kizomba Parejas</v>
       </c>
       <c r="G3" t="str">
-        <v>SOFIA</v>
+        <v>FABI</v>
       </c>
       <c r="H3" t="str">
         <v>OK</v>
@@ -3383,109 +3543,103 @@
         <v>20000.00</v>
       </c>
       <c r="J3" t="str">
-        <v>2025-04-01</v>
+        <v>2025-03-01</v>
       </c>
       <c r="K3" t="str">
-        <v>2025-08-31</v>
+        <v>2025-07-31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Clase kizomba</v>
+        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
       </c>
       <c r="B4">
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
       <c r="C4" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango</v>
       </c>
       <c r="D4" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango (Inter/Avanz)</v>
       </c>
       <c r="E4" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
       </c>
       <c r="F4" t="str">
-        <v>Coreográfico Femenino</v>
+        <v>Tango</v>
       </c>
       <c r="G4" t="str">
-        <v>SOFIA</v>
+        <v>ROBERTO</v>
       </c>
       <c r="H4" t="str">
-        <v>NOT_A_TARIFF</v>
+        <v>OK</v>
       </c>
       <c r="I4" t="str">
-        <v>21000.00</v>
+        <v>15000.00</v>
       </c>
       <c r="J4" t="str">
-        <v>2025-09-01</v>
+        <v>2025-02-01</v>
       </c>
       <c r="K4" t="str">
-        <v>2025-09-30</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Importe particular o condición especial; no representa la tarifa general.</v>
+        <v>2025-02-28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Clase kizomba</v>
+        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
       </c>
       <c r="B5">
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
       <c r="C5" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango</v>
       </c>
       <c r="D5" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango (Inter/Avanz)</v>
       </c>
       <c r="E5" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
       </c>
       <c r="F5" t="str">
-        <v>Coreográfico Femenino</v>
+        <v>Tango</v>
       </c>
       <c r="G5" t="str">
-        <v>SOFIA</v>
+        <v>ROBERTO</v>
       </c>
       <c r="H5" t="str">
-        <v>NOT_A_TARIFF</v>
+        <v>OK</v>
       </c>
       <c r="I5" t="str">
-        <v>30000.00</v>
+        <v>20000.00</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-02-01</v>
+        <v>2025-03-01</v>
       </c>
       <c r="K5" t="str">
-        <v>2026-03-31</v>
-      </c>
-      <c r="L5" t="str">
-        <v>La academia confirmó cuota general de $30.000 entre enero y abril de 2026; $15.000 fue un importe especial.</v>
+        <v>2025-08-31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Clase kizomba</v>
+        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
       </c>
       <c r="B6">
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
       <c r="C6" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango</v>
       </c>
       <c r="D6" t="str">
-        <v>Clase femenino Sofi</v>
+        <v>Tango (Inter/Avanz)</v>
       </c>
       <c r="E6" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
+        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
       </c>
       <c r="F6" t="str">
-        <v>Coreográfico Femenino</v>
+        <v>Tango</v>
       </c>
       <c r="G6" t="str">
-        <v>SOFIA</v>
+        <v>ROBERTO</v>
       </c>
       <c r="H6" t="str">
         <v>OK</v>
@@ -3494,842 +3648,25 @@
         <v>30000.00</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-05-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-06-30</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B7">
-        <v>0.25</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="E7" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Coreográfico Femenino</v>
-      </c>
-      <c r="G7" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="H7" t="str">
-        <v>NOT_A_TARIFF</v>
-      </c>
-      <c r="I7" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="J7" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="K7" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Medio mes o condición especial</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B8">
-        <v>0.25</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="E8" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Coreográfico Femenino</v>
-      </c>
-      <c r="G8" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="H8" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I8" t="str">
-        <v>40000.00</v>
-      </c>
-      <c r="J8" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="K8" t="str">
-        <v>2026-08-31</v>
-      </c>
-      <c r="L8" t="str">
-        <v>La academia confirmó que desde agosto de 2026 la cuota normal pasó a $40.000.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B9">
-        <v>0.25</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="E9" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Estilo Femenino</v>
-      </c>
-      <c r="G9" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="H9" t="str">
-        <v>NOT_A_TARIFF</v>
-      </c>
-      <c r="I9" t="str">
-        <v>7500.00</v>
-      </c>
-      <c r="J9" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="K9" t="str">
-        <v>2025-02-28</v>
-      </c>
-      <c r="L9" t="str">
-        <v>La academia confirmó que la cuota general de febrero de 2025 era $15.000; $7.500 correspondía a una condición especial.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B10">
-        <v>0.25</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="E10" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Estilo Femenino</v>
-      </c>
-      <c r="G10" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="H10" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I10" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="J10" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="K10" t="str">
-        <v>2025-08-31</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B11">
-        <v>0.25</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="E11" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Estilo Femenino</v>
-      </c>
-      <c r="G11" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="H11" t="str">
-        <v>NOT_A_TARIFF</v>
-      </c>
-      <c r="I11" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="J11" t="str">
-        <v>2025-09-01</v>
-      </c>
-      <c r="K11" t="str">
-        <v>2025-10-31</v>
-      </c>
-      <c r="L11" t="str">
-        <v>Importe particular o condición especial; no representa la tarifa general.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
-      </c>
-      <c r="B12">
-        <v>0.5</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Ritmos Caribeños y Kizomba Parejas</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Ritmos latinos y caribeños</v>
-      </c>
-      <c r="E12" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Ritmos Caribeños y Kizomba Parejas</v>
-      </c>
-      <c r="G12" t="str">
-        <v>FABI</v>
-      </c>
-      <c r="H12" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I12" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="J12" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="K12" t="str">
-        <v>2025-02-28</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
-      </c>
-      <c r="B13">
-        <v>0.5</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Ritmos Caribeños y Kizomba Parejas</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Ritmos latinos y caribeños</v>
-      </c>
-      <c r="E13" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Ritmos Caribeños y Kizomba Parejas</v>
-      </c>
-      <c r="G13" t="str">
-        <v>FABI</v>
-      </c>
-      <c r="H13" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I13" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="J13" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="K13" t="str">
-        <v>2025-07-31</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Grupo C. Sofi</v>
-      </c>
-      <c r="B14">
-        <v>0.4</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Grupo C. - A.Frank</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Grupo C. - A.Frank</v>
-      </c>
-      <c r="E14" t="str">
-        <v>e63b18a1-afc2-4fd1-aa80-dfce8909e30f</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Estilo Frank</v>
-      </c>
-      <c r="G14" t="str">
-        <v>ANA</v>
-      </c>
-      <c r="H14" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I14" t="str">
-        <v>25000.00</v>
-      </c>
-      <c r="J14" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="K14" t="str">
-        <v>2026-03-31</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Grupo C. Sofi</v>
-      </c>
-      <c r="B15">
-        <v>0.4</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Grupo C. - A.Frank</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Grupo C. - A.Frank</v>
-      </c>
-      <c r="E15" t="str">
-        <v>e63b18a1-afc2-4fd1-aa80-dfce8909e30f</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Estilo Frank</v>
-      </c>
-      <c r="G15" t="str">
-        <v>ANA</v>
-      </c>
-      <c r="H15" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I15" t="str">
-        <v>25000.00</v>
-      </c>
-      <c r="J15" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="K15" t="str">
-        <v>2026-06-30</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="B16">
-        <v>0.286</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="E16" t="str">
-        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="G16" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="H16" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I16" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="J16" t="str">
-        <v>2025-05-01</v>
-      </c>
-      <c r="K16" t="str">
-        <v>2025-05-31</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="B17">
-        <v>0.286</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="E17" t="str">
-        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="G17" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="H17" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I17" t="str">
-        <v>10000.00</v>
-      </c>
-      <c r="J17" t="str">
-        <v>2025-06-01</v>
-      </c>
-      <c r="K17" t="str">
-        <v>2025-06-30</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="B18">
-        <v>0.286</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="E18" t="str">
-        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="G18" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="H18" t="str">
-        <v>NOT_A_TARIFF</v>
-      </c>
-      <c r="I18" t="str">
-        <v>5000.00</v>
-      </c>
-      <c r="J18" t="str">
-        <v>2025-07-01</v>
-      </c>
-      <c r="K18" t="str">
-        <v>2025-07-31</v>
-      </c>
-      <c r="L18" t="str">
-        <v>Condición especial definida por el profesor</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="B19">
-        <v>0.6</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="E19" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="G19" t="str">
-        <v>ROBERTO</v>
-      </c>
-      <c r="H19" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I19" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="J19" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="K19" t="str">
-        <v>2025-02-28</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="B20">
-        <v>0.6</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="E20" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="G20" t="str">
-        <v>ROBERTO</v>
-      </c>
-      <c r="H20" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I20" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="J20" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="K20" t="str">
-        <v>2025-08-31</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="B21">
-        <v>0.6</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="E21" t="str">
-        <v>cc392129-75e3-4205-b7fc-fafceb55b996</v>
-      </c>
-      <c r="F21" t="str">
-        <v>Tango</v>
-      </c>
-      <c r="G21" t="str">
-        <v>ROBERTO</v>
-      </c>
-      <c r="H21" t="str">
-        <v>OK</v>
-      </c>
-      <c r="I21" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="J21" t="str">
-        <v>2025-09-01</v>
-      </c>
-      <c r="K21" t="str">
         <v>2025-11-30</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Clase objetivo</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Score</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Clase candidata</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Class ID candidato</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Importe</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Desde</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Hasta</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B2">
-        <v>0.25</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D2" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E2" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="F2" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2025-02-28</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B3">
-        <v>0.25</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D3" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E3" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2025-09-30</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B4">
-        <v>0.25</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D4" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E4" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="F4" t="str">
-        <v>2025-10-01</v>
-      </c>
-      <c r="G4" t="str">
-        <v>2025-10-31</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B5">
-        <v>0.25</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D5" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E5" t="str">
-        <v>25000.00</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2025-11-01</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-02-28</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B6">
-        <v>0.25</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D6" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E6" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-07-31</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Clase kizomba</v>
-      </c>
-      <c r="B7">
-        <v>0.25</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D7" t="str">
-        <v>d0762bb4-c6ef-45d4-8414-5ae0f158831f</v>
-      </c>
-      <c r="E7" t="str">
-        <v>40000.00</v>
-      </c>
-      <c r="F7" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="G7" t="str">
-        <v>2026-08-31</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
-      </c>
-      <c r="B8">
-        <v>0.375</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Ritmos latinos y caribeños</v>
-      </c>
-      <c r="D8" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
-      </c>
-      <c r="E8" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="G8" t="str">
-        <v>2025-02-28</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
-      </c>
-      <c r="B9">
-        <v>0.375</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Ritmos latinos y caribeños</v>
-      </c>
-      <c r="D9" t="str">
-        <v>1a8e1c0e-1f96-4de2-a33d-c932e74f2314</v>
-      </c>
-      <c r="E9" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="F9" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="G9" t="str">
-        <v>2025-07-31</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Grupo C. Sofi</v>
-      </c>
-      <c r="B10">
-        <v>0.4</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Grupo C. - A.Frank</v>
-      </c>
-      <c r="D10" t="str">
-        <v>e63b18a1-afc2-4fd1-aa80-dfce8909e30f</v>
-      </c>
-      <c r="E10" t="str">
-        <v>25000.00</v>
-      </c>
-      <c r="F10" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="G10" t="str">
-        <v>2026-06-30</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="B11">
-        <v>0.286</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="D11" t="str">
-        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
-      </c>
-      <c r="E11" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="F11" t="str">
-        <v>2025-05-01</v>
-      </c>
-      <c r="G11" t="str">
-        <v>2025-05-31</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="B12">
-        <v>0.286</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="D12" t="str">
-        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
-      </c>
-      <c r="E12" t="str">
-        <v>10000.00</v>
-      </c>
-      <c r="F12" t="str">
-        <v>2025-06-01</v>
-      </c>
-      <c r="G12" t="str">
-        <v>2025-06-30</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6797,15 +6134,15 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>NO_SOURCE_EVIDENCE</v>
+        <v>CONFIRMED_MAPPING</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>WORKBOOK_EVIDENCE_ONLY</v>
+        <v>CONFIRMED_HISTORICAL_ACTIVITY</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -6813,15 +6150,15 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>POSSIBLE_ALIAS</v>
+        <v>CONFIRMED_SPECIAL_PROGRAM</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SPECIAL_PROGRAM_REVIEW</v>
+        <v>TEST_CLASS</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -6891,4 +6228,999 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M24"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Clase actual</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Class ID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Tipo mapping</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Nombre histórico confirmado</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Profesor</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tarifa base</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Política tarifaria</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actividad encontrada</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Resultado analysis</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Importe</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Desde</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Hasta</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Motivo</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>S&amp;B Parejas</v>
+      </c>
+      <c r="B2" t="str">
+        <v>576c192b-8d45-47e9-bd94-df027445d793</v>
+      </c>
+      <c r="C2" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Salsa y Bachata en Pareja | Salsa Y Bachata En Pareja | Salsa Y Bachata En Pareja _Fabi</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>PO confirmó que S&amp;B Parejas corresponde a Salsa y Bachata en Pareja.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Clase kizomba</v>
+      </c>
+      <c r="B3" t="str">
+        <v>b9c792eb-ea2e-47f5-b436-f6cfe5c5ac26</v>
+      </c>
+      <c r="C3" t="str">
+        <v>HISTORICAL_ACTIVITY</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Kizomba | Clase Kizomba</v>
+      </c>
+      <c r="E3" t="str">
+        <v>FABI</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>GENERAL_ACADEMY_RATE</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>PO confirmó que corresponde a la clase de Kizomba de Fabi y utilizaba la cuota base general de la academia.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Hells</v>
+      </c>
+      <c r="B4" t="str">
+        <v>0dd78cf5-7a17-455c-9a70-1175a12d327d</v>
+      </c>
+      <c r="C4" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Heels</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>PO confirmó que Hells es un error de escritura y corresponde a Heels.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Formacion Docente En Ritmos Caribeños Y Kizomba</v>
+      </c>
+      <c r="B5" t="str">
+        <v>50f07573-4f58-4314-a0aa-e2e2d0feae71</v>
+      </c>
+      <c r="C5" t="str">
+        <v>SPECIAL_PROGRAM</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Formacion Docente En Ritmos Caribeños Y Kizomba | Formación Docente En Ritmos Caribeños Y Kizomba</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>90000.00</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>PO confirmó que la formación comenzó en abril de 2026, termina en diciembre de 2026 y tiene cuota base mensual de $90.000. Los valores $76.500, $72.000 y becas son condiciones particulares.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E6" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I6" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J6" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2025-02-01</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2025-02-28</v>
+      </c>
+      <c r="M6" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B7" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C7" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E7" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I7" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J7" t="str">
+        <v>20000.00</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2025-04-01</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2025-08-31</v>
+      </c>
+      <c r="M7" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C8" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E8" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I8" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J8" t="str">
+        <v>21000.00</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2025-09-01</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2025-09-30</v>
+      </c>
+      <c r="M8" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I9" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J9" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="M9" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E10" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I10" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J10" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="M10" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C11" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E11" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I11" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J11" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="M11" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C12" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="E12" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Coreográfico Femenino</v>
+      </c>
+      <c r="I12" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J12" t="str">
+        <v>40000.00</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="M12" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B13" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C13" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E13" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I13" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J13" t="str">
+        <v>7500.00</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2025-02-01</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2025-02-28</v>
+      </c>
+      <c r="M13" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C14" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E14" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I14" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J14" t="str">
+        <v>20000.00</v>
+      </c>
+      <c r="K14" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2025-08-31</v>
+      </c>
+      <c r="M14" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B15" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C15" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E15" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I15" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J15" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="K15" t="str">
+        <v>2025-09-01</v>
+      </c>
+      <c r="L15" t="str">
+        <v>2025-10-31</v>
+      </c>
+      <c r="M15" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B16" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E16" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I16" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J16" t="str">
+        <v>25000.00</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2025-11-01</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2025-11-30</v>
+      </c>
+      <c r="M16" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B17" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C17" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E17" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I17" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J17" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="K17" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="L17" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="M17" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C18" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E18" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I18" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J18" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="K18" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="M18" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B19" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C19" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E19" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I19" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J19" t="str">
+        <v>30000.00</v>
+      </c>
+      <c r="K19" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="L19" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="M19" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C20" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E20" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I20" t="str">
+        <v>NOT_A_TARIFF</v>
+      </c>
+      <c r="J20" t="str">
+        <v>15000.00</v>
+      </c>
+      <c r="K20" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="M20" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Grupo C. Sofi</v>
+      </c>
+      <c r="B21" t="str">
+        <v>ac972b45-74ce-49f8-be10-3a6f0151da82</v>
+      </c>
+      <c r="C21" t="str">
+        <v>SAME_ACTIVITY</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="E21" t="str">
+        <v>SOFIA</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>Estilo Femenino</v>
+      </c>
+      <c r="I21" t="str">
+        <v>OK</v>
+      </c>
+      <c r="J21" t="str">
+        <v>40000.00</v>
+      </c>
+      <c r="K21" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L21" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="M21" t="str">
+        <v>PO confirmó que Grupo C. Sofi corresponde al Coreográfico Femenino de Sofi.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Coreografico E.Masc-Bachata/Urban</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2d17175b-22b0-4565-9342-1e93ad221855</v>
+      </c>
+      <c r="C22" t="str">
+        <v>HISTORICAL_ACTIVITY</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Coreografico E Masc Bachata Urban | Coreográfico E Masc Bachata Urban | Coreografico E.Masc-Bachata/Urban</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>GENERAL_ACADEMY_RATE</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v>PO confirmó que era una actividad independiente, utilizaba la cuota general y posteriormente pasó a llamarse Urban Flow.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>arabashe</v>
+      </c>
+      <c r="B23" t="str">
+        <v>ff270dd4-aef0-4546-aeb7-24aa94093098</v>
+      </c>
+      <c r="C23" t="str">
+        <v>TEST_CLASS</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v>Clase de prueba. No corresponde reconstruir tarifas históricas y será eliminada posteriormente.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
+      </c>
+      <c r="B24" t="str">
+        <v>7b64e0e6-a347-4734-b2fa-b752fbe92cfb</v>
+      </c>
+      <c r="C24" t="str">
+        <v>SPECIAL_PROGRAM</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Inst Sup Coreografico Tango 18 Meses | Inst.Sup.Coreografico -Tango /18 Meses | Instituto Superior Coreografico Tango 18 Meses</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>70000.00</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v>PO confirmó que era un programa diferente de Tango regular, con cuota mensual de $70.000 y actualmente está dado de baja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M24"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>